<commit_message>
Deployed 9266e0d with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/anexos/md03/lista_piezas_estructura.xlsx
+++ b/anexos/md03/lista_piezas_estructura.xlsx
@@ -18,6 +18,7 @@
     <definedName name="Movev_Final_componentes_Extructura_y_Base_v7" localSheetId="0">Hoja1!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -245,14 +246,16 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -262,8 +265,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Énfasis5" xfId="1" builtinId="46"/>
@@ -562,266 +563,266 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="H1" s="7" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="H1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="9"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="11"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="4"/>
+      <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>1800</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>4</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <f>C3*D3/1000</f>
         <v>7.2</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="5">
         <f>SUMIF($B:$B, H3, $E:$E)*1.05</f>
         <v>17.682000000000002</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="5">
         <f>ROUNDUP(I3/6,0)</f>
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>300</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>2</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <f t="shared" ref="E4:E12" si="0">C4*D4/1000</f>
         <v>0.6</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="6">
-        <f t="shared" ref="I4:I6" si="1">SUMIF($B:$B, H4, $E:$E)*1.05</f>
+      <c r="I4" s="5">
+        <f>SUMIF($B:$B, H4, $E:$E)*1.05</f>
         <v>8.2467000000000006</v>
       </c>
-      <c r="J4" s="6">
-        <f t="shared" ref="J4:J6" si="2">ROUNDUP(I4/6,0)</f>
+      <c r="J4" s="5">
+        <f>ROUNDUP(I4/6,0)</f>
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>600</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>7</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="6">
-        <f t="shared" si="1"/>
+      <c r="I5" s="5">
+        <f>SUMIF($B:$B, H5, $E:$E)*1.05</f>
         <v>1.3776000000000002</v>
       </c>
-      <c r="J5" s="6">
-        <f t="shared" si="2"/>
+      <c r="J5" s="5">
+        <f>ROUNDUP(I5/6,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>310</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>4</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <f t="shared" si="0"/>
         <v>1.24</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="6">
-        <f t="shared" si="1"/>
+      <c r="I6" s="5">
+        <f>SUMIF($B:$B, H6, $E:$E)*1.05</f>
         <v>0.52500000000000002</v>
       </c>
-      <c r="J6" s="6">
-        <f t="shared" si="2"/>
+      <c r="J6" s="5">
+        <f>ROUNDUP(I6/6,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>266</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>2</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <f t="shared" si="0"/>
         <v>0.53200000000000003</v>
       </c>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>337</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>2</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <f t="shared" si="0"/>
         <v>0.67400000000000004</v>
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>302</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>4</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <f t="shared" si="0"/>
         <v>1.208</v>
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>250</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>2</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>656</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>2</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <f t="shared" si="0"/>
         <v>1.3120000000000001</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <v>565</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>16</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="2">
         <f t="shared" si="0"/>
         <v>9.0399999999999991</v>
       </c>

</xml_diff>